<commit_message>
refactor(transferencias): el campo de procedencia se volvio en text, se hizo el cambio en todo el sistema
</commit_message>
<xml_diff>
--- a/resources/templates/plantilla_transferencia_2026.xlsx
+++ b/resources/templates/plantilla_transferencia_2026.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\servidor\laragon\www\sistema_archivo\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E09DFC2-E7DA-47D6-B64E-13368A967835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF8D2F48-4638-4E56-884D-E0A9234F10E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{18BFF21B-825A-45FF-AB6E-B8F0BA73624E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{18BFF21B-825A-45FF-AB6E-B8F0BA73624E}"/>
   </bookViews>
   <sheets>
     <sheet name="TRANSFERENCIA" sheetId="3" r:id="rId1"/>
     <sheet name="AYUDAS" sheetId="5" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TRANSFERENCIA!$A$5:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TRANSFERENCIA!$A$5:$J$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="52">
   <si>
     <t>CORRESPONDENCIA</t>
   </si>
@@ -67,9 +67,6 @@
     <t>CODIGO DE REFERENCIA</t>
   </si>
   <si>
-    <t>PROCEDENCIA</t>
-  </si>
-  <si>
     <t>DESCRIPCION DOCUMENTAL (LOMO)</t>
   </si>
   <si>
@@ -109,18 +106,6 @@
     <t>REGLAMENTO ESPECIFICO DEL SISTEMA DE ADMINISTRACION DE PERSONAL</t>
   </si>
   <si>
-    <t>SGM,AGJAM,AJAM</t>
-  </si>
-  <si>
-    <t>SGM</t>
-  </si>
-  <si>
-    <t>AJAM</t>
-  </si>
-  <si>
-    <t>AGJAM</t>
-  </si>
-  <si>
     <t>2005-2006</t>
   </si>
   <si>
@@ -275,53 +260,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>1/16</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Registre la sigla correspondiente a la procedencia. Las siglas válidas se encuentran en la hoja </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PARAMETRICAS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Cuando exista más de una procedencia, sepárelas mediante coma, por ejemplo: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SGM,AGJAM</t>
     </r>
     <r>
       <rPr>
@@ -521,7 +459,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,12 +494,6 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -649,7 +581,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -676,9 +608,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -692,9 +621,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -722,10 +648,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1060,368 +986,343 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F93B41C-3457-4549-A41A-2244B0E67E6E}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="55.77734375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="55.77734375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="13" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="19.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18.5546875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="28.6640625" style="5" customWidth="1"/>
-    <col min="12" max="16384" width="11.44140625" style="2"/>
+    <col min="3" max="3" width="19.77734375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="55.77734375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="55.77734375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="13" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="28.6640625" style="5" customWidth="1"/>
+    <col min="11" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="32" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="32" t="s">
+      <c r="B2" s="28"/>
+      <c r="C2" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="33" t="s">
+      <c r="B3" s="29"/>
+      <c r="C3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-    </row>
-    <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+    </row>
+    <row r="4" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="B4" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K4" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>35</v>
+      <c r="B5" s="20" t="s">
+        <v>30</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="9">
+        <v>1</v>
+      </c>
+      <c r="G5" s="11">
+        <v>12</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="14">
+        <v>2</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="14">
+        <v>1</v>
+      </c>
+      <c r="G6" s="16">
+        <v>32</v>
+      </c>
+      <c r="H6" s="17">
+        <v>2001</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="14">
+        <v>3</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="14">
+        <v>1</v>
+      </c>
+      <c r="G7" s="16">
+        <v>20</v>
+      </c>
+      <c r="H7" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="I7" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="14">
+        <v>4</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="D8" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="14">
+        <v>1</v>
+      </c>
+      <c r="G8" s="16">
+        <v>75</v>
+      </c>
+      <c r="H8" s="17">
+        <v>2005</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="14">
+        <v>5</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="14">
+        <v>1</v>
+      </c>
+      <c r="G9" s="16">
+        <v>25</v>
+      </c>
+      <c r="H9" s="17">
+        <v>2008</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="14">
+        <v>6</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="14">
+        <v>1</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="9">
-        <v>1</v>
-      </c>
-      <c r="H5" s="12">
-        <v>12</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="K5" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" s="14" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15">
-        <v>2</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="17" t="s">
+      <c r="H10" s="17">
+        <v>2008</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="J10" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="15">
-        <v>1</v>
-      </c>
-      <c r="H6" s="18">
-        <v>32</v>
-      </c>
-      <c r="I6" s="19">
-        <v>2001</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="15">
-        <v>3</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="15">
-        <v>1</v>
-      </c>
-      <c r="H7" s="18">
-        <v>20</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="K7" s="20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="45.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="15">
-        <v>4</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="15">
-        <v>1</v>
-      </c>
-      <c r="H8" s="18">
-        <v>75</v>
-      </c>
-      <c r="I8" s="19">
-        <v>2005</v>
-      </c>
-      <c r="J8" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="15">
-        <v>5</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" s="15">
-        <v>1</v>
-      </c>
-      <c r="H9" s="18">
-        <v>25</v>
-      </c>
-      <c r="I9" s="19">
-        <v>2008</v>
-      </c>
-      <c r="J9" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="K9" s="20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="15">
-        <v>6</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="G10" s="15">
-        <v>1</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="I10" s="19">
-        <v>2008</v>
-      </c>
-      <c r="J10" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="K10" s="20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="21"/>
-    </row>
-    <row r="12" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
-    </row>
-    <row r="13" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
-    </row>
-    <row r="14" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-    </row>
-    <row r="15" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-    </row>
-    <row r="16" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
+    </row>
+    <row r="11" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B11" s="19"/>
+    </row>
+    <row r="12" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B12" s="19"/>
+    </row>
+    <row r="13" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B13" s="19"/>
+    </row>
+    <row r="14" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B14" s="19"/>
+    </row>
+    <row r="15" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B15" s="19"/>
+    </row>
+    <row r="16" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B16" s="19"/>
     </row>
     <row r="17" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
+      <c r="B17" s="19"/>
     </row>
     <row r="18" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B18" s="21"/>
+      <c r="B18" s="19"/>
     </row>
     <row r="19" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
+      <c r="B19" s="19"/>
     </row>
     <row r="20" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B20" s="21"/>
+      <c r="B20" s="19"/>
     </row>
     <row r="21" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B21" s="21"/>
+      <c r="B21" s="19"/>
     </row>
     <row r="22" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B22" s="21"/>
+      <c r="B22" s="19"/>
     </row>
     <row r="23" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B23" s="21"/>
+      <c r="B23" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C1:K1"/>
-    <mergeCell ref="C2:K2"/>
-    <mergeCell ref="C3:K3"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.19685039370078741" bottom="0.23622047244094491" header="0.19685039370078741" footer="0.23622047244094491"/>
   <pageSetup scale="60" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -1430,131 +1331,123 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{241D6D74-CF70-4C06-A326-3763228D5ABF}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="73.44140625" style="25" customWidth="1"/>
+    <col min="2" max="2" width="73.44140625" style="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="26" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="26" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="28" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="26" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="28" t="s">
+    <row r="9" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="26" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="28" t="s">
+    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="26" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="28" t="s">
+    <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="26" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="28" t="s">
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="26" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="27" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="28" t="s">
+    <row r="13" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="26" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="28" t="s">
+    <row r="14" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="26" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="28" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="28" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>